<commit_message>
paper run 2026-10-08 10:32
</commit_message>
<xml_diff>
--- a/reports/2026-10-08.xlsx
+++ b/reports/2026-10-08.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,92 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-08T07:11:19.642684+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F2" t="n">
+        <v>56.02</v>
+      </c>
+      <c r="G2" t="n">
+        <v>109.84</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.00107</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>53.82</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-08T09:26:18.466648+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00117</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>18.4</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -536,6 +622,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>72.22</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>72.22</v>
       </c>
     </row>
     <row r="8">
@@ -573,6 +662,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2806.179999999998</v>
+        <v>2878.399999999999</v>
       </c>
     </row>
     <row r="12">
@@ -628,114 +720,181 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>457.31</v>
+      </c>
+      <c r="E15" t="n">
+        <v>72.22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По активам</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>129.51</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>327.8</v>
+      </c>
+      <c r="E18" t="n">
+        <v>72.22</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>384.11</v>
+      </c>
+      <c r="E20" t="n">
+        <v>72.22</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>202.71</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>254.6</v>
+      </c>
+      <c r="E24" t="n">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -744,45 +903,223 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>72.22</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>53.82</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>18.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="n">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>72.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-08 18:36
</commit_message>
<xml_diff>
--- a/reports/2026-10-08.xlsx
+++ b/reports/2026-10-08.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,393 @@
       </c>
       <c r="K3" t="n">
         <v>18.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-08T13:56:15.870297+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="G4" t="n">
+        <v>114.76</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.00161</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>50.49</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-08T15:38:48.269732+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5393</v>
+      </c>
+      <c r="F5" t="n">
+        <v>20.28</v>
+      </c>
+      <c r="G5" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.819</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.00304</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>17.32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-08T15:41:22.130846+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00129</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>8.800000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-08T15:48:46.162503+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00126</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-08T16:41:25.271017+00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.00184</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-08T17:09:15.532101+00:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="G9" t="n">
+        <v>14</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.00144</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>6.02</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-08T17:13:08.305058+00:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F10" t="n">
+        <v>81.19</v>
+      </c>
+      <c r="G10" t="n">
+        <v>150.36</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.802</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>69.17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-08T17:43:17.194142+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="G11" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-0.00183</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-08T18:11:16.754965+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-0.00188</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>-4.48</v>
       </c>
     </row>
   </sheetData>
@@ -571,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,7 +980,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -603,7 +990,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -613,7 +1000,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -623,7 +1010,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0.8181818181818182</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +1020,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>72.22</v>
+        <v>224.49</v>
       </c>
     </row>
     <row r="7">
@@ -643,7 +1030,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>72.22</v>
+        <v>234.97</v>
       </c>
     </row>
     <row r="8">
@@ -653,7 +1040,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>-10.48</v>
       </c>
     </row>
     <row r="9">
@@ -663,7 +1050,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>99</v>
+        <v>22.42</v>
       </c>
     </row>
     <row r="10">
@@ -673,7 +1060,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2878.399999999999</v>
+        <v>3030.669999999999</v>
       </c>
     </row>
     <row r="12">
@@ -724,294 +1111,329 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>457.31</v>
+        <v>1519.6</v>
       </c>
       <c r="E15" t="n">
-        <v>72.22</v>
+        <v>207.15</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>460.4</v>
+      </c>
+      <c r="E16" t="n">
+        <v>17.34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>129.51</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>327.8</v>
+        <v>112.29</v>
       </c>
       <c r="E18" t="n">
-        <v>72.22</v>
+        <v>50.49</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>313.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
-        <v>384.11</v>
+        <v>633.55</v>
       </c>
       <c r="E20" t="n">
-        <v>72.22</v>
+        <v>107.78</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>73.2</v>
+        <v>920.36</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>66.22</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
+          <t>По цене входа</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D23" t="n">
-        <v>202.71</v>
+        <v>1255.67</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>158.71</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
-        <v>254.6</v>
+        <v>463.94</v>
       </c>
       <c r="E24" t="n">
-        <v>72.22</v>
+        <v>56.03</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>260.39</v>
+      </c>
+      <c r="E25" t="n">
+        <v>9.75</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" t="n">
+        <v>277.27</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D28" t="n">
+        <v>950.51</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C29" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>72.22</v>
+        <v>752.22</v>
+      </c>
+      <c r="E29" t="n">
+        <v>224.49</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" t="n">
-        <v>72.22</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>50.49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
-        <v>53.82</v>
+        <v>107.78</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>18.4</v>
+        <v>66.22</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1033,93 +1455,377 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" t="n">
+        <v>7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>207.15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" t="n">
         <v>2</v>
       </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="n">
-        <v>72.22</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+      <c r="D40" t="n">
+        <v>17.34</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" t="n">
-        <v>72.22</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>53.82</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>18.4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>50.49</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>20.12</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D48" t="n">
+        <v>84.94</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-4.48</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="n">
+        <v>158.71</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6</v>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>56.03</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>72.22</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3</v>
+      </c>
+      <c r="D58" t="n">
+        <v>77.98999999999999</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>56.96</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>17.32</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="n">
+        <v>-0.73</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>2</v>
-      </c>
-      <c r="C45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" t="n">
-        <v>72.22</v>
+      <c r="B64" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" t="n">
+        <v>8</v>
+      </c>
+      <c r="D64" t="n">
+        <v>225.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>